<commit_message>
feat: add mappings for UKSL, ATC, and DNFBP watchlists
</commit_message>
<xml_diff>
--- a/data/rules/preNormalization.xlsx
+++ b/data/rules/preNormalization.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hajibashi.Saba\Desktop\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2F59452-08AA-4C73-A967-04F3DE800C15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC022FBF-399D-4111-AE70-67F56243C981}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{664D7B0B-3A54-AB4A-9B2E-0F6BCF1A0441}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="37">
   <si>
     <t>source</t>
   </si>
@@ -61,13 +61,7 @@
     <t>Individual</t>
   </si>
   <si>
-    <t>Organization</t>
-  </si>
-  <si>
     <t>Vessel</t>
-  </si>
-  <si>
-    <t>Entity=Organization</t>
   </si>
   <si>
     <t>OFAC-SDN</t>
@@ -89,9 +83,6 @@
   </si>
   <si>
     <t>sanctionsLists.sanctionsList.text</t>
-  </si>
-  <si>
-    <t>generalInfo.entityType.text</t>
   </si>
   <si>
     <t>relationships.relationship[].type.text</t>
@@ -141,14 +132,43 @@
   <si>
     <t>Primary Name=primary Name|Alias=AKA</t>
   </si>
+  <si>
+    <t xml:space="preserve">Entity </t>
+  </si>
+  <si>
+    <t>DNFBP</t>
+  </si>
+  <si>
+    <t>UPDATING OF REGISTRATION IS REQUIRED ON</t>
+  </si>
+  <si>
+    <t>date_format</t>
+  </si>
+  <si>
+    <t>MM/DD/YYYY</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -205,9 +225,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -530,11 +556,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD38AAAA-71AD-464E-BCF4-8B613DCBC998}">
-  <dimension ref="A1:AA996"/>
+  <dimension ref="A1:AA993"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="29.83203125" customWidth="1"/>
-    <col min="3" max="3" width="39.1640625" customWidth="1"/>
+    <col min="3" max="3" width="45.33203125" customWidth="1"/>
     <col min="4" max="4" width="29.33203125" customWidth="1"/>
     <col min="5" max="5" width="92.5" customWidth="1"/>
   </cols>
@@ -580,19 +606,19 @@
     </row>
     <row r="2" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="3" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>6</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>
@@ -619,19 +645,19 @@
     </row>
     <row r="3" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="3" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>6</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
@@ -658,19 +684,19 @@
     </row>
     <row r="4" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="3" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>6</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="F4" s="3"/>
       <c r="G4" s="3"/>
@@ -697,19 +723,19 @@
     </row>
     <row r="5" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>6</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
@@ -736,19 +762,19 @@
     </row>
     <row r="6" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>6</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
@@ -775,19 +801,19 @@
     </row>
     <row r="7" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>6</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
@@ -814,16 +840,16 @@
     </row>
     <row r="8" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
@@ -851,16 +877,16 @@
     </row>
     <row r="9" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
@@ -888,16 +914,16 @@
     </row>
     <row r="10" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
@@ -925,19 +951,19 @@
     </row>
     <row r="11" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A11" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>6</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
@@ -964,19 +990,19 @@
     </row>
     <row r="12" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A12" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>6</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F12" s="3"/>
       <c r="G12" s="3"/>
@@ -1003,20 +1029,18 @@
     </row>
     <row r="13" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
-      <c r="E13" s="3" t="s">
-        <v>10</v>
-      </c>
+      <c r="E13" s="3"/>
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
@@ -1042,16 +1066,16 @@
     </row>
     <row r="14" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
-      <c r="B14" s="3" t="s">
-        <v>7</v>
+      <c r="B14" s="4" t="s">
+        <v>32</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
@@ -1078,19 +1102,21 @@
       <c r="AA14" s="3"/>
     </row>
     <row r="15" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="3" t="s">
-        <v>16</v>
+      <c r="A15" s="1" t="s">
+        <v>19</v>
       </c>
-      <c r="B15" s="3" t="s">
-        <v>8</v>
+      <c r="B15" s="1" t="s">
+        <v>22</v>
       </c>
-      <c r="C15" s="3" t="s">
-        <v>21</v>
+      <c r="C15" s="1" t="s">
+        <v>23</v>
       </c>
-      <c r="D15" s="3" t="s">
-        <v>20</v>
+      <c r="D15" s="1" t="s">
+        <v>6</v>
       </c>
-      <c r="E15" s="3"/>
+      <c r="E15" s="1" t="s">
+        <v>24</v>
+      </c>
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
       <c r="H15" s="3"/>
@@ -1115,17 +1141,17 @@
       <c r="AA15" s="3"/>
     </row>
     <row r="16" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="3" t="s">
-        <v>16</v>
+      <c r="A16" s="1" t="s">
+        <v>19</v>
       </c>
-      <c r="B16" s="3" t="s">
-        <v>9</v>
+      <c r="B16" s="1" t="s">
+        <v>7</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D16" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>20</v>
       </c>
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
@@ -1152,20 +1178,20 @@
       <c r="AA16" s="3"/>
     </row>
     <row r="17" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A17" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B17" s="1" t="s">
+      <c r="A17" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="B17" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C17" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D17" s="1" t="s">
+      <c r="D17" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E17" s="1" t="s">
-        <v>27</v>
+      <c r="E17" s="3" t="s">
+        <v>28</v>
       </c>
       <c r="F17" s="3"/>
       <c r="G17" s="3"/>
@@ -1191,19 +1217,21 @@
       <c r="AA17" s="3"/>
     </row>
     <row r="18" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A18" s="1" t="s">
+      <c r="A18" t="s">
+        <v>33</v>
+      </c>
+      <c r="B18" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B18" s="1" t="s">
-        <v>7</v>
+      <c r="C18" t="s">
+        <v>34</v>
       </c>
-      <c r="C18" s="1" t="s">
-        <v>23</v>
+      <c r="D18" t="s">
+        <v>35</v>
       </c>
-      <c r="D18" s="1" t="s">
-        <v>24</v>
+      <c r="E18" t="s">
+        <v>36</v>
       </c>
-      <c r="E18" s="3"/>
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
       <c r="H18" s="3"/>
@@ -1228,21 +1256,11 @@
       <c r="AA18" s="3"/>
     </row>
     <row r="19" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A19" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>10</v>
-      </c>
+      <c r="A19" s="3"/>
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
       <c r="H19" s="3"/>
@@ -1267,21 +1285,11 @@
       <c r="AA19" s="3"/>
     </row>
     <row r="20" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A20" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>31</v>
-      </c>
+      <c r="A20" s="3"/>
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
       <c r="H20" s="3"/>
@@ -29522,93 +29530,6 @@
       <c r="Z993" s="3"/>
       <c r="AA993" s="3"/>
     </row>
-    <row r="994" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A994" s="3"/>
-      <c r="B994" s="3"/>
-      <c r="C994" s="3"/>
-      <c r="D994" s="3"/>
-      <c r="E994" s="3"/>
-      <c r="F994" s="3"/>
-      <c r="G994" s="3"/>
-      <c r="H994" s="3"/>
-      <c r="I994" s="3"/>
-      <c r="J994" s="3"/>
-      <c r="K994" s="3"/>
-      <c r="L994" s="3"/>
-      <c r="M994" s="3"/>
-      <c r="N994" s="3"/>
-      <c r="O994" s="3"/>
-      <c r="P994" s="3"/>
-      <c r="Q994" s="3"/>
-      <c r="R994" s="3"/>
-      <c r="S994" s="3"/>
-      <c r="T994" s="3"/>
-      <c r="U994" s="3"/>
-      <c r="V994" s="3"/>
-      <c r="W994" s="3"/>
-      <c r="X994" s="3"/>
-      <c r="Y994" s="3"/>
-      <c r="Z994" s="3"/>
-      <c r="AA994" s="3"/>
-    </row>
-    <row r="995" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A995" s="3"/>
-      <c r="B995" s="3"/>
-      <c r="C995" s="3"/>
-      <c r="D995" s="3"/>
-      <c r="E995" s="3"/>
-      <c r="F995" s="3"/>
-      <c r="G995" s="3"/>
-      <c r="H995" s="3"/>
-      <c r="I995" s="3"/>
-      <c r="J995" s="3"/>
-      <c r="K995" s="3"/>
-      <c r="L995" s="3"/>
-      <c r="M995" s="3"/>
-      <c r="N995" s="3"/>
-      <c r="O995" s="3"/>
-      <c r="P995" s="3"/>
-      <c r="Q995" s="3"/>
-      <c r="R995" s="3"/>
-      <c r="S995" s="3"/>
-      <c r="T995" s="3"/>
-      <c r="U995" s="3"/>
-      <c r="V995" s="3"/>
-      <c r="W995" s="3"/>
-      <c r="X995" s="3"/>
-      <c r="Y995" s="3"/>
-      <c r="Z995" s="3"/>
-      <c r="AA995" s="3"/>
-    </row>
-    <row r="996" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A996" s="3"/>
-      <c r="B996" s="3"/>
-      <c r="C996" s="3"/>
-      <c r="D996" s="3"/>
-      <c r="E996" s="3"/>
-      <c r="F996" s="3"/>
-      <c r="G996" s="3"/>
-      <c r="H996" s="3"/>
-      <c r="I996" s="3"/>
-      <c r="J996" s="3"/>
-      <c r="K996" s="3"/>
-      <c r="L996" s="3"/>
-      <c r="M996" s="3"/>
-      <c r="N996" s="3"/>
-      <c r="O996" s="3"/>
-      <c r="P996" s="3"/>
-      <c r="Q996" s="3"/>
-      <c r="R996" s="3"/>
-      <c r="S996" s="3"/>
-      <c r="T996" s="3"/>
-      <c r="U996" s="3"/>
-      <c r="V996" s="3"/>
-      <c r="W996" s="3"/>
-      <c r="X996" s="3"/>
-      <c r="Y996" s="3"/>
-      <c r="Z996" s="3"/>
-      <c r="AA996" s="3"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
fix(postnorm): make date_order config required so it can't be silently dropped
</commit_message>
<xml_diff>
--- a/data/rules/preNormalization.xlsx
+++ b/data/rules/preNormalization.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hajibashi.Saba\Desktop\python-components\data\rules\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC022FBF-399D-4111-AE70-67F56243C981}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E80DBF8-4AAB-4D17-9255-A1A96E2C05C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{664D7B0B-3A54-AB4A-9B2E-0F6BCF1A0441}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="33">
   <si>
     <t>source</t>
   </si>
@@ -134,18 +134,6 @@
   </si>
   <si>
     <t xml:space="preserve">Entity </t>
-  </si>
-  <si>
-    <t>DNFBP</t>
-  </si>
-  <si>
-    <t>UPDATING OF REGISTRATION IS REQUIRED ON</t>
-  </si>
-  <si>
-    <t>date_format</t>
-  </si>
-  <si>
-    <t>MM/DD/YYYY</t>
   </si>
 </sst>
 </file>
@@ -1217,21 +1205,7 @@
       <c r="AA17" s="3"/>
     </row>
     <row r="18" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A18" t="s">
-        <v>33</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="C18" t="s">
-        <v>34</v>
-      </c>
-      <c r="D18" t="s">
-        <v>35</v>
-      </c>
-      <c r="E18" t="s">
-        <v>36</v>
-      </c>
+      <c r="B18" s="5"/>
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
       <c r="H18" s="3"/>

</xml_diff>

<commit_message>
feat(names): split SECO spelling variants into per-name Original Script + Language
</commit_message>
<xml_diff>
--- a/data/rules/preNormalization.xlsx
+++ b/data/rules/preNormalization.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42C1BBBF-567F-40A0-BD51-F4283C5F49FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{626DBCE6-C4C9-47D4-B4B4-70A82E3AC34C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="51">
   <si>
     <t>source</t>
   </si>
@@ -149,6 +149,30 @@
   </si>
   <si>
     <t>INDIVIDUAL=Individual|ENTITY=Entity</t>
+  </si>
+  <si>
+    <t>Target type</t>
+  </si>
+  <si>
+    <t>PERSON=Individual|ORGANISATION=Entity|SCHIFF=Vessel</t>
+  </si>
+  <si>
+    <t>Other information</t>
+  </si>
+  <si>
+    <t>regex_extract</t>
+  </si>
+  <si>
+    <t>(?i)IMO\s*Numbe?r?\D*(\d+)</t>
+  </si>
+  <si>
+    <t>Spelling variants</t>
+  </si>
+  <si>
+    <t>split_pattern</t>
+  </si>
+  <si>
+    <t>(?P&lt;name&gt;.+?)(?P&lt;_translit&gt;(?&lt;=[^\x00-\x7F])\s+[A-Za-z][A-Za-z0-9 .,'’-]*)?\s*\((?P&lt;language&gt;[^()]+)\)\s*$</t>
   </si>
 </sst>
 </file>
@@ -1372,11 +1396,21 @@
       <c r="AA21" s="3"/>
     </row>
     <row r="22" spans="1:27" ht="35.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A22" s="3"/>
-      <c r="B22" s="3"/>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
-      <c r="E22" s="5"/>
+      <c r="A22" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>44</v>
+      </c>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
       <c r="H22" s="3"/>
@@ -1401,11 +1435,21 @@
       <c r="AA22" s="3"/>
     </row>
     <row r="23" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A23" s="3"/>
-      <c r="B23" s="3"/>
-      <c r="C23" s="3"/>
-      <c r="D23" s="3"/>
-      <c r="E23" s="3"/>
+      <c r="A23" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>47</v>
+      </c>
       <c r="F23" s="3"/>
       <c r="G23" s="3"/>
       <c r="H23" s="3"/>
@@ -1430,11 +1474,21 @@
       <c r="AA23" s="3"/>
     </row>
     <row r="24" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A24" s="3"/>
-      <c r="B24" s="3"/>
-      <c r="C24" s="3"/>
-      <c r="D24" s="3"/>
-      <c r="E24" s="3"/>
+      <c r="A24" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>50</v>
+      </c>
       <c r="F24" s="3"/>
       <c r="G24" s="3"/>
       <c r="H24" s="3"/>

</xml_diff>

<commit_message>
feat(PDG-3): de-quote FBI aliases in pre-normalization
</commit_message>
<xml_diff>
--- a/data/rules/preNormalization.xlsx
+++ b/data/rules/preNormalization.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{626DBCE6-C4C9-47D4-B4B4-70A82E3AC34C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB25A140-230B-4E46-97A8-F0A43CF03B4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="54">
   <si>
     <t>source</t>
   </si>
@@ -173,6 +173,15 @@
   </si>
   <si>
     <t>(?P&lt;name&gt;.+?)(?P&lt;_translit&gt;(?&lt;=[^\x00-\x7F])\s+[A-Za-z][A-Za-z0-9 .,'’-]*)?\s*\((?P&lt;language&gt;[^()]+)\)\s*$</t>
+  </si>
+  <si>
+    <t>FBI-WANTED</t>
+  </si>
+  <si>
+    <t>aliases[]</t>
+  </si>
+  <si>
+    <t>^"?(.*?)"?$</t>
   </si>
 </sst>
 </file>
@@ -1513,11 +1522,21 @@
       <c r="AA24" s="3"/>
     </row>
     <row r="25" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A25" s="3"/>
-      <c r="B25" s="3"/>
-      <c r="C25" s="3"/>
-      <c r="D25" s="3"/>
-      <c r="E25" s="3"/>
+      <c r="A25" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>53</v>
+      </c>
       <c r="F25" s="3"/>
       <c r="G25" s="3"/>
       <c r="H25" s="3"/>

</xml_diff>

<commit_message>
feat(PDG-22): finalize INTERPOL Red Notices mapping and language-name handler
- add language_name pre-normalization handler: ISO 639-2/B code -> English language name via pycountry; unresolvable/collective codes (CAU, DRA) and nulls pass through unchanged

- retune INTERPOL faceting order (null-free axes first: name, forename, arrestWarrantCountryId, then nationality) for faster planning

- onboard INTERPOL-RED-NOTICES into the conformance and golden suites with a 50-record sample fixture

- mapping.xlsx also carries a new declared-but-unrouted 'Aircraft' entity category (not used by INTERPOL); guard updated to tolerate it as the two share one xlsx binary
</commit_message>
<xml_diff>
--- a/data/rules/preNormalization.xlsx
+++ b/data/rules/preNormalization.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D6AFE68-2DB9-42A1-8E89-630E551472BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88103BC8-0003-4C1B-BE72-D02FF41F5A6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="70">
   <si>
     <t>source</t>
   </si>
@@ -204,14 +204,48 @@
   <si>
     <t>True=Active|False=Inactive</t>
   </si>
+  <si>
+    <t>INTERPOL-RED-NOTICES</t>
+  </si>
+  <si>
+    <t>detail.sex_id</t>
+  </si>
+  <si>
+    <t>M=Male|F=Female|U=Unknown</t>
+  </si>
+  <si>
+    <t>detail.eyes_colors_id[]</t>
+  </si>
+  <si>
+    <t>BLA=Black|BLU=Blue|BLUL=Light Blue|BRO=Brown|BROD=Dark Brown|BROL=Light Brown|BROH=Hazel|GRE=Green|GRY=Grey|OTHD=Other (Dark)|OTHL=Other (Light)</t>
+  </si>
+  <si>
+    <t>detail.hairs_id[]</t>
+  </si>
+  <si>
+    <t>BLA=Black|BRO=Brown|BROL=Light Brown|BROF=Fair Brown|GRY=Grey|GRYG=Greying|RED=Red|REDA=Auburn|WHI=White|YELB=Blond|YELBD=Dark Blond|HAIB=Bald|HAID=Balding|OTHD=Other (Dark)</t>
+  </si>
+  <si>
+    <t>detail.languages_spoken_ids[]</t>
+  </si>
+  <si>
+    <t>language_name</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -288,9 +322,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -299,23 +336,23 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1681,11 +1718,21 @@
       <c r="AA27" s="3"/>
     </row>
     <row r="28" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A28" s="3"/>
-      <c r="B28" s="3"/>
-      <c r="C28" s="3"/>
-      <c r="D28" s="3"/>
-      <c r="E28" s="3"/>
+      <c r="A28" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>63</v>
+      </c>
       <c r="F28" s="3"/>
       <c r="G28" s="3"/>
       <c r="H28" s="3"/>
@@ -1709,12 +1756,22 @@
       <c r="Z28" s="3"/>
       <c r="AA28" s="3"/>
     </row>
-    <row r="29" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A29" s="3"/>
-      <c r="B29" s="3"/>
-      <c r="C29" s="3"/>
-      <c r="D29" s="3"/>
-      <c r="E29" s="3"/>
+    <row r="29" spans="1:27" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A29" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>65</v>
+      </c>
       <c r="F29" s="3"/>
       <c r="G29" s="3"/>
       <c r="H29" s="3"/>
@@ -1738,12 +1795,22 @@
       <c r="Z29" s="3"/>
       <c r="AA29" s="3"/>
     </row>
-    <row r="30" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A30" s="3"/>
-      <c r="B30" s="3"/>
-      <c r="C30" s="3"/>
-      <c r="D30" s="3"/>
-      <c r="E30" s="3"/>
+    <row r="30" spans="1:27" ht="29.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A30" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>67</v>
+      </c>
       <c r="F30" s="3"/>
       <c r="G30" s="3"/>
       <c r="H30" s="3"/>
@@ -1768,10 +1835,18 @@
       <c r="AA30" s="3"/>
     </row>
     <row r="31" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A31" s="3"/>
-      <c r="B31" s="3"/>
-      <c r="C31" s="3"/>
-      <c r="D31" s="3"/>
+      <c r="A31" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C31" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="D31" s="11" t="s">
+        <v>69</v>
+      </c>
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
       <c r="G31" s="3"/>

</xml_diff>

<commit_message>
feat(PDG-37): onboard US Marshals Profiled Fugitives watchlist
Add the source yaml and watchlist config (akamai bypass crawler), the mapping.xlsx column and preNormalization rules, and a hashed source_record_id via generate_composite_id (also applied to INTERPOL). Add a 50-record sample fixture and register the list in the golden and conformance suites.
</commit_message>
<xml_diff>
--- a/data/rules/preNormalization.xlsx
+++ b/data/rules/preNormalization.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88103BC8-0003-4C1B-BE72-D02FF41F5A6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C526F9B7-8B41-401A-A794-4CFB4B32FB34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1520" yWindow="1520" windowWidth="15680" windowHeight="9430" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="75">
   <si>
     <t>source</t>
   </si>
@@ -231,14 +231,36 @@
   <si>
     <t>language_name</t>
   </si>
+  <si>
+    <t>US-MARSHALS-PROFILED-FUGITIVES</t>
+  </si>
+  <si>
+    <t>attachments[].type</t>
+  </si>
+  <si>
+    <t>detail.height</t>
+  </si>
+  <si>
+    <t>^([^"]*)</t>
+  </si>
+  <si>
+    <t>IMAGE=Photograph|DOCUMENT=Poster|DETAIL_PAGE=Other|THUMBNAIL=Thumbnail</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -322,9 +344,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -333,23 +358,23 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1872,11 +1897,21 @@
       <c r="AA31" s="3"/>
     </row>
     <row r="32" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A32" s="3"/>
-      <c r="B32" s="3"/>
-      <c r="C32" s="3"/>
-      <c r="D32" s="3"/>
-      <c r="E32" s="3"/>
+      <c r="A32" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E32" s="12" t="s">
+        <v>74</v>
+      </c>
       <c r="F32" s="3"/>
       <c r="G32" s="3"/>
       <c r="H32" s="3"/>
@@ -1901,11 +1936,21 @@
       <c r="AA32" s="3"/>
     </row>
     <row r="33" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A33" s="3"/>
-      <c r="B33" s="3"/>
-      <c r="C33" s="3"/>
-      <c r="D33" s="3"/>
-      <c r="E33" s="3"/>
+      <c r="A33" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>73</v>
+      </c>
       <c r="F33" s="3"/>
       <c r="G33" s="3"/>
       <c r="H33" s="3"/>

</xml_diff>